<commit_message>
fix: timezone + admin notification + stock at 20:20
- gsheet_db, appointment_db: _now_iso() ใช้ Asia/Bangkok เสมอ
  (Railway = UTC → registration timestamps เคยเป็น UTC แล้วเพี้ยน 7 ชม.)
- chatbot_server: เพิ่ม bkk_now() helper + แก้ thai_date_short() / get_today_appointments()
- appointment_sender: notify_admin_presend ใช้ LOVELY_BOT_TOKEN (ของ Wirote)
  แทน LINE_OA_TOKEN ที่ Wirote ไม่เป็นเพื่อน + เช็ค HTTP status ก่อน print success
- scheduler.run_daily_summary: ส่ง stock message แยกที่ hour==20 (รอบ 20:20)
- chatbot_server./run_summary_now: รองรับ ?stock=1 และ stock auto ที่ hour==20

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/appointments.xlsx
+++ b/appointments.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:54</t>
+          <t>2026-05-26 21:05:09</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:54</t>
+          <t>2026-05-26 21:05:10</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:55</t>
+          <t>2026-05-26 21:05:11</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:56</t>
+          <t>2026-05-26 21:05:12</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:57</t>
+          <t>2026-05-26 21:05:13</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:58</t>
+          <t>2026-05-26 21:05:14</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-26 20:37:59</t>
+          <t>2026-05-26 21:05:15</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-26 20:38:00</t>
+          <t>2026-05-26 21:05:15</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-26 20:38:00</t>
+          <t>2026-05-26 21:05:16</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:08</t>
+          <t>2026-05-26 21:05:17</t>
         </is>
       </c>
     </row>
@@ -964,6 +964,9 @@
           <t>พัมกิ้น</t>
         </is>
       </c>
+      <c r="F14" t="n">
+        <v>954486615</v>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>2026-05-26 20:36:35</t>
@@ -971,7 +974,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:09</t>
+          <t>2026-05-26 21:05:18</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1006,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:10</t>
+          <t>2026-05-26 21:05:19</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1018,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>690299-1</t>
+          <t>690299-3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1025,7 +1028,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>บราวนี่</t>
+          <t>ส้มจิ๋ว</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1035,7 +1038,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:11</t>
+          <t>2026-05-26 21:05:20</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1070,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:12</t>
+          <t>2026-05-26 21:05:21</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1102,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:13</t>
+          <t>2026-05-26 21:05:22</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1134,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-05-26 20:40:14</t>
+          <t>2026-05-26 21:05:23</t>
         </is>
       </c>
     </row>
@@ -1325,6 +1328,85 @@
         </is>
       </c>
       <c r="I24" t="inlineStr">
+        <is>
+          <t>auto_sibling</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>U47aa79494e18e479471bae5f420f8caf</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>690299-1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ณัฐวิญญ์ สิรเดชธราทิพย์</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>บราวนี่</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:30:15</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:30:15</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>auto_sibling</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>U22ef391387145f0f1cfd0889a2e437f9</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>690084-3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>แนน</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ชาไทย</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0660146423</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-05-27 20:15:12</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-05-27 20:15:12</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>auto_sibling</t>
         </is>
@@ -1341,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1416,37 +1498,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DRX-577</t>
+          <t>DRX-300</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>690276-1</t>
+          <t>690162-1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>หญิง</t>
+          <t>นุชอนงค์ กุลกิตติโกวิท</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>วอดก้า</t>
+          <t>ชาเย็น</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ,รับยาต่อเนื่อง</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1456,44 +1538,44 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DRX-613</t>
+          <t>DRX-301</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>690001-1</t>
+          <t>690162-1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tarn Tarn.</t>
+          <t>นุชอนงค์ กุลกิตติโกวิท</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>หมูกะทะ</t>
+          <t>ชาเย็น</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (โทร)</t>
+          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/2) + พิษสุนัขบ้า (2/2))</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1503,44 +1585,44 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DRX-615</t>
+          <t>DRX-309</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>690001-1</t>
+          <t>690007-1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tarn Tarn.</t>
+          <t>สุชาวดี ชาติกานนท์</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>หมูกะทะ</t>
+          <t>มันนี่</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — อื่นๆ (Ngsp)</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1550,44 +1632,44 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DRX-538</t>
+          <t>DRX-295</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>690239-1</t>
+          <t>690159-1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>นิลภวิษย์ ทับทอง</t>
+          <t>พรพรรณ ณัฐวุฒิ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ฟ้า</t>
+          <t>หมูแดง</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ฉีดวัคซีน — วัคซีนไข้หัดและหวัดแมว (วัคซีน,ถ่ายพยาธิ,หยดยา,ดูอาการขา)</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1597,44 +1679,44 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DRX-560</t>
+          <t>DRX-303</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>690001-1</t>
+          <t>690162-2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tarn Tarn.</t>
+          <t>นุชอนงค์ กุลกิตติโกวิท</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>หมูกะทะ</t>
+          <t>สแกมเมอร์</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ให้น้ำเกลือ</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1644,44 +1726,44 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DRX-585</t>
+          <t>DRX-304</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>690224-1</t>
+          <t>690162-2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>มัลลิณี ศรีจันทร์</t>
+          <t>นุชอนงค์ กุลกิตติโกวิท</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>คิรัว</t>
+          <t>สแกมเมอร์</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — X-ray</t>
+          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/2)+ พิษสุนัข (2/2))</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1691,44 +1773,44 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DRX-612</t>
+          <t>DRX-568</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>690001-1</t>
+          <t>690241-1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tarn Tarn.</t>
+          <t>สุทธินันท์ มุสิกาวัน</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>หมูกะทะ</t>
+          <t>ชีต้า</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>สัตวแพทย์</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — X-ray</t>
+          <t>ตรวจทั่วไป — โทรถามอาการเรื่องคันหู</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1738,29 +1820,29 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DRX-614</t>
+          <t>DRX-586</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>690001-1</t>
+          <t>690224-1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tarn Tarn.</t>
+          <t>มัลลิณี ศรีจันทร์</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>หมูกะทะ</t>
+          <t>คิรัว</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1770,12 +1852,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (โทรถาม)</t>
+          <t>ตรวจทั่วไป — Ultrasound</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1785,29 +1867,29 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DRX-641</t>
+          <t>DRX-617</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>690296-1</t>
+          <t>690291-1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>รต ไพศาล อิศรางกูร</t>
+          <t>ธนิตา ถวิลวิสา</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>เจี๊ยบ</t>
+          <t>จากัวร์</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1817,12 +1899,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — โทรสอบถามเรื่องคลอด</t>
+          <t>ตรวจทั่วไป — โทรสอบถามอาการถ่ายเหลว</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1832,29 +1914,29 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DRX-300</t>
+          <t>DRX-621</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>690162-1</t>
+          <t>690293-1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>นุชอนงค์ กุลกิตติโกวิท</t>
+          <t>สริตา ปรึกษากร</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ชาเย็น</t>
+          <t>มีเธอ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1864,7 +1946,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — โทรสอบอาการ</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1879,44 +1961,44 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DRX-301</t>
+          <t>DRX-587</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>690162-1</t>
+          <t>690224-1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>นุชอนงค์ กุลกิตติโกวิท</t>
+          <t>มัลลิณี ศรีจันทร์</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ชาเย็น</t>
+          <t>คิรัว</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/2) + พิษสุนัขบ้า (2/2))</t>
+          <t>ตรวจทั่วไป — ตรวจเลือด</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1926,44 +2008,44 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DRX-561</t>
+          <t>DRX-645</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>690277-1</t>
+          <t>690257-1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>อภิญญา สุขใจ</t>
+          <t>สุณิสา</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>อวกาศ</t>
+          <t>โชคดี</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ,ตรวจเลือด (cbc)</t>
+          <t>ตรวจทั่วไป — ฉีดยา (ฉีด EPO)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1973,44 +2055,44 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DRX-309</t>
+          <t>DRX-592</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>690007-1</t>
+          <t>690278-1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>สุชาวดี ชาติกานนท์</t>
+          <t>สุทธิ เข้มกำเนิด</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>มันนี่</t>
+          <t>ทอง</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>สัตวแพทย์</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ดูอาการ</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2020,44 +2102,44 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DRX-647</t>
+          <t>DRX-639</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>690289-1</t>
+          <t>690280-1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>นัฒริยา เลี้ยงอำนวย</t>
+          <t>คณิติน ยวนแหล</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>แมวส้ม</t>
+          <t>จิ๋ว</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>เบญจมาศ</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ทำแผล,ฉีดยา</t>
+          <t>ตรวจทั่วไป — ทำแผล</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2067,29 +2149,29 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DRX-295</t>
+          <t>DRX-663</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>690159-1</t>
+          <t>690289-1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>พรพรรณ ณัฐวุฒิ</t>
+          <t>นัฒริยา เลี้ยงอำนวย</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>หมูแดง</t>
+          <t>แมวส้ม</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2099,12 +2181,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ทำแผล,ฉีดยา</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2114,44 +2196,44 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DRX-299</t>
+          <t>DRX-320</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>690160-1</t>
+          <t>690171-2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ธนากร เจริญธนารัตน์</t>
+          <t>สุดารัตน์ โพธิ์ทอง</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>โพเนีย</t>
+          <t>ไดม่อน</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>มัลลินี</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (3/3) + พิษสุนัขบ้า (2/2))</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2161,29 +2243,29 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DRX-303</t>
+          <t>DRX-321</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>690162-2</t>
+          <t>690171-2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>นุชอนงค์ กุลกิตติโกวิท</t>
+          <t>สุดารัตน์ โพธิ์ทอง</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>สแกมเมอร์</t>
+          <t>ไดม่อน</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2193,12 +2275,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2208,29 +2290,29 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DRX-304</t>
+          <t>DRX-323</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>690162-2</t>
+          <t>690171-1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>นุชอนงค์ กุลกิตติโกวิท</t>
+          <t>สุดารัตน์ โพธิ์ทอง</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>สแกมเมอร์</t>
+          <t>ดราก้อน (แพคเกจวัคซีน)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2240,12 +2322,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/2)+ พิษสุนัข (2/2))</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2255,44 +2337,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DRX-564</t>
+          <t>DRX-329</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>690130-1</t>
+          <t>690178-1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>กานดา ตันติสกุลเลิศ</t>
+          <t>ณิชจิรา เติมสินสวัสดิ์</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>คุมะ</t>
+          <t>มะยม (แพคเกจวัคซีน)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — รับยาต่อเนื่อง (โทรถามอาการ + รับยาต่อเนื่อง)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2302,44 +2384,44 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DRX-568</t>
+          <t>DRX-322</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>690241-1</t>
+          <t>690171-1</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>สุทธินันท์ มุสิกาวัน</t>
+          <t>สุดารัตน์ โพธิ์ทอง</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ชีต้า</t>
+          <t>ดราก้อน (แพคเกจวัคซีน)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — โทรถามอาการเรื่องคันหู</t>
+          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/3) +  พิษสุนัขบ้า (1/2))</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2349,44 +2431,44 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DRX-586</t>
+          <t>DRX-328</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>690224-1</t>
+          <t>690178-1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>มัลลิณี ศรีจันทร์</t>
+          <t>ณิชจิรา เติมสินสวัสดิ์</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>คิรัว</t>
+          <t>มะยม (แพคเกจวัคซีน)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — Ultrasound</t>
+          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/3) + พิษสุนัขบ้า (2/2))</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2396,44 +2478,44 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DRX-617</t>
+          <t>DRX-589</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>690291-1</t>
+          <t>690284-1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ธนิตา ถวิลวิสา</t>
+          <t>จันทนี เซี่ยงคิ้ว</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>จากัวร์</t>
+          <t>ชานม</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>สัตวแพทย์</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — โทรสอบถามอาการถ่ายเหลว</t>
+          <t>ตรวจทั่วไป — ดูอาการ,รับยาต่อเนื่อง</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2443,44 +2525,44 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DRX-621</t>
+          <t>DRX-600</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>690293-1</t>
+          <t>690136-1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>สริตา ปรึกษากร</t>
+          <t>ลูกนัท</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>มีเธอ</t>
+          <t>มีอาร์</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>สัตวแพทย์</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — โทรสอบอาการ</t>
+          <t>ตรวจทั่วไป — ดูอาการ (+/- กระตุ้นวัคซีน รวม2/2 + RV2/2)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2490,44 +2572,44 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DRX-587</t>
+          <t>DRX-638</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>690224-1</t>
+          <t>690295-1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>มัลลิณี ศรีจันทร์</t>
+          <t>สุพรรษา วิโอประเสริฐ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>คิรัว</t>
+          <t>กะทิ</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ตรวจเลือด</t>
+          <t>ตรวจทั่วไป — โทรสอบถามอาการไอ</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2537,29 +2619,29 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DRX-645</t>
+          <t>DRX-643</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>690257-1</t>
+          <t>690298-1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>สุณิสา</t>
+          <t>กรรณิการ์ วุฒิกุล</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>โชคดี</t>
+          <t>มาตังค์</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2569,12 +2651,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ฉีดยา (ฉีด EPO)</t>
+          <t>ตรวจทั่วไป — ดูอาการ (ตาบวม)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2584,44 +2666,44 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DRX-592</t>
+          <t>DRX-644</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>690278-1</t>
+          <t>690152-4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>สุทธิ เข้มกำเนิด</t>
+          <t>ปวริศ มากสอน</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ทอง</t>
+          <t>บีน่า</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ</t>
+          <t>ตรวจทั่วไป — ดูอาการ (เท้าบวม)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2631,44 +2713,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DRX-639</t>
+          <t>DRX-606</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>690280-1</t>
+          <t>690287-1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>คณิติน ยวนแหล</t>
+          <t>กิ่งกมล เรืองหิรัญ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>จิ๋ว</t>
+          <t>ไก่ตุ๋น</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>เบญจมาศ</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ทำแผล</t>
+          <t>ตรวจทั่วไป — ดูอาการ (ระบบประสาท)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2678,29 +2760,29 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DRX-320</t>
+          <t>DRX-651</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>690171-2</t>
+          <t>690201-1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>สุดารัตน์ โพธิ์ทอง</t>
+          <t>ปรารถนา ไวปัญญา</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ไดม่อน</t>
+          <t>เหมย (แพคเกจวัคซีน)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2710,12 +2792,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (3/3) + พิษสุนัขบ้า (2/2))</t>
+          <t>ตรวจทั่วไป — ดูอาการ (ฟอกเชื้อรา + รับยาต่อเนื่อง)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2725,29 +2807,29 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DRX-321</t>
+          <t>DRX-602</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>690171-2</t>
+          <t>690206-2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>สุดารัตน์ โพธิ์ทอง</t>
+          <t>สุฐิษา ธนาการกิตติสุข</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ไดม่อน</t>
+          <t>นีออน</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2757,12 +2839,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ดูอาการ (โทรสอบถามอาการ)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2772,29 +2854,29 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DRX-323</t>
+          <t>DRX-618</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>690171-1</t>
+          <t>690291-1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>สุดารัตน์ โพธิ์ทอง</t>
+          <t>ธนิตา ถวิลวิสา</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ดราก้อน (แพคเกจวัคซีน)</t>
+          <t>จากัวร์</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2804,12 +2886,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ดูอาการ (+/- ทำวัคซีนเข็มแรก)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2819,29 +2901,29 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DRX-329</t>
+          <t>DRX-622</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>690178-1</t>
+          <t>690293-1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ณิชจิรา เติมสินสวัสดิ์</t>
+          <t>สริตา ปรึกษากร</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>มะยม (แพคเกจวัคซีน)</t>
+          <t>มีเธอ</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2851,12 +2933,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
+          <t>ตรวจทั่วไป — ดูอาการ (+/- วัคซีนเข็มแรก)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2866,44 +2948,44 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DRX-322</t>
+          <t>DRX-516</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>690171-1</t>
+          <t>690092-1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>สุดารัตน์ โพธิ์ทอง</t>
+          <t>ธนภรณ์</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ดราก้อน (แพคเกจวัคซีน)</t>
+          <t>ทองมา</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>มัลลินี</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/3) +  พิษสุนัขบ้า (1/2))</t>
+          <t>ตรวจทั่วไป — ดูอาการ (ตรวจตา)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2913,29 +2995,29 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DRX-328</t>
+          <t>DRX-357</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>690178-1</t>
+          <t>690196-1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ณิชจิรา เติมสินสวัสดิ์</t>
+          <t>อนัญญา เทียนธนะวัฒธ์</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>มะยม (แพคเกจวัคซีน)</t>
+          <t>ฮันนี่</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2945,12 +3027,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/3) + พิษสุนัขบ้า (2/2))</t>
+          <t>ตรวจทั่วไป — X-ray</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2960,44 +3042,44 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DRX-589</t>
+          <t>DRX-664</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>690284-1</t>
+          <t>690302-1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>จันทนี เซี่ยงคิ้ว</t>
+          <t>ธัญสินี กาญจนสิทธิ์</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ชานม</t>
+          <t>คาฟู</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ,รับยาต่อเนื่อง</t>
+          <t>ตรวจทั่วไป — ตัดไหม</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3007,44 +3089,44 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DRX-600</t>
+          <t>DRX-64</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>690136-1</t>
+          <t>690038-2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ลูกนัท</t>
+          <t>วริทธ์นานนท์ ขจิตศาตนันท์</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>มีอาร์</t>
+          <t>ขุมทรัพย์</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>สัตวแพทย์</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (+/- กระตุ้นวัคซีน รวม2/2 + RV2/2)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3054,29 +3136,29 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DRX-638</t>
+          <t>DRX-65</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>690295-1</t>
+          <t>690038-1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>สุพรรษา วิโอประเสริฐ</t>
+          <t>วริทธ์นานนท์ ขจิตศาตนันท์</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>กะทิ</t>
+          <t>โยดา</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3086,12 +3168,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — โทรสอบถามอาการไอ</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3101,44 +3183,44 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DRX-643</t>
+          <t>DRX-69</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>690298-1</t>
+          <t>690043-1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>กรรณิการ์ วุฒิกุล</t>
+          <t>รื่นรมย์ เหรียญทอง</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>มาตังค์</t>
+          <t>สองสี</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (ตาบวม)</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก (DW)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3148,44 +3230,44 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DRX-644</t>
+          <t>DRX-81</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>690152-4</t>
+          <t>690039-1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ปวริศ มากสอน</t>
+          <t>อาร์ม</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>บีน่า</t>
+          <t>สาคู</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (เท้าบวม)</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก (DW)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3195,29 +3277,29 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DRX-606</t>
+          <t>DRX-85</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>690287-1</t>
+          <t>690026-2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>กิ่งกมล เรืองหิรัญ</t>
+          <t>ญานิศา แรงจันทร์</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ไก่ตุ๋น</t>
+          <t>ชิโร่ (แพคเกจวัคซีน)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3227,12 +3309,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (ระบบประสาท)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ (DW)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3242,44 +3324,44 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DRX-651</t>
+          <t>DRX-87</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>690201-1</t>
+          <t>690056-1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ปรารถนา ไวปัญญา</t>
+          <t>อรธิมา เอกจีน</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>เหมย (แพคเกจวัคซีน)</t>
+          <t>ไอโชค</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (ฟอกเชื้อรา + รับยาต่อเนื่อง)</t>
+          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก (BVT,DW)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3289,29 +3371,29 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DRX-602</t>
+          <t>DRX-110</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>690206-2</t>
+          <t>690067-1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>สุฐิษา ธนาการกิตติสุข</t>
+          <t>ไก่</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>นีออน</t>
+          <t>อั่งเปา</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3321,12 +3403,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (โทรสอบถามอาการ)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3336,29 +3418,29 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DRX-618</t>
+          <t>DRX-117</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>690291-1</t>
+          <t>690072-1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ธนิตา ถวิลวิสา</t>
+          <t>ปิ่นแก้ว</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>จากัวร์</t>
+          <t>มาโร</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3368,12 +3450,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (+/- ทำวัคซีนเข็มแรก)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3383,29 +3465,29 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DRX-622</t>
+          <t>DRX-126</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>690293-1</t>
+          <t>690076-1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>สริตา ปรึกษากร</t>
+          <t>อรพรรณ  ขำสุวรรณ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>มีเธอ</t>
+          <t>น้องถุงเงิน</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3415,12 +3497,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (+/- วัคซีนเข็มแรก)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3430,44 +3512,44 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DRX-516</t>
+          <t>DRX-142</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>690092-1</t>
+          <t>690082-1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ธนภรณ์</t>
+          <t>ประชุม คุณท้าวเทียม</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ทองมา</t>
+          <t>มีบุญ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>มัลลินี</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ดูอาการ (ตรวจตา)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3477,29 +3559,29 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DRX-357</t>
+          <t>DRX-151</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>690196-1</t>
+          <t>690096-1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>อนัญญา เทียนธนะวัฒธ์</t>
+          <t>กฤตยา วิเชียรพาย</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ฮันนี่</t>
+          <t>ซาร่า</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3509,12 +3591,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — X-ray</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3524,29 +3606,29 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DRX-64</t>
+          <t>DRX-161</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>690038-2</t>
+          <t>690100-1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>วริทธ์นานนท์ ขจิตศาตนันท์</t>
+          <t>พิสิทธิ์    สามกองงาม</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ขุมทรัพย์</t>
+          <t>กิมจิ</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3561,7 +3643,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3571,29 +3653,29 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DRX-65</t>
+          <t>DRX-159</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>690038-1</t>
+          <t>690100-2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>วริทธ์นานนท์ ขจิตศาตนันท์</t>
+          <t>พิสิทธิ์    สามกองงาม</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>โยดา</t>
+          <t>โซจู</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3608,7 +3690,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3618,44 +3700,44 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DRX-69</t>
+          <t>DRX-163</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>690043-1</t>
+          <t>690056-2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>รื่นรมย์ เหรียญทอง</t>
+          <t>อรธิมา เอกจีน</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>สองสี</t>
+          <t>เฉาก๊วย</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก (DW)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3665,44 +3747,44 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DRX-81</t>
+          <t>DRX-164</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>690039-1</t>
+          <t>690056-3</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>อาร์ม</t>
+          <t>อรธิมา เอกจีน</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>สาคู</t>
+          <t>พาดกลอน</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก (DW)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3712,29 +3794,29 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DRX-85</t>
+          <t>DRX-174</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>690026-2</t>
+          <t>690056-4</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ญานิศา แรงจันทร์</t>
+          <t>อรธิมา เอกจีน</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ชิโร่ (แพคเกจวัคซีน)</t>
+          <t>บี1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3744,12 +3826,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ (DW)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3759,44 +3841,44 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DRX-87</t>
+          <t>DRX-180</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>690056-1</t>
+          <t>690042-2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>อรธิมา เอกจีน</t>
+          <t>วราฤทธิ์ บัวโต</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ไอโชค</t>
+          <t>ดั๊ก</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>โรงพยาบาลสัตว์หมาแมวเลิฟลี่</t>
+          <t>นารีรัตน์ ผลทิพย์</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก (BVT,DW)</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3806,29 +3888,29 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DRX-110</t>
+          <t>DRX-172</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>690067-1</t>
+          <t>690056-5</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ไก่</t>
+          <t>อรธิมา เอกจีน</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>อั่งเปา</t>
+          <t>บี2</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3843,7 +3925,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3853,29 +3935,29 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DRX-117</t>
+          <t>DRX-191</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>690072-1</t>
+          <t>690009-6</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ปิ่นแก้ว</t>
+          <t>ธนาวดี เมธา</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>มาโร</t>
+          <t>ปลาหมึก</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3890,7 +3972,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3900,29 +3982,29 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DRX-126</t>
+          <t>DRX-210</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>690076-1</t>
+          <t>690064-2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>อรพรรณ  ขำสุวรรณ</t>
+          <t>จีรวรรณ มณีโชติ</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>น้องถุงเงิน</t>
+          <t>พลูโต</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3937,7 +4019,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3947,29 +4029,29 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DRX-142</t>
+          <t>DRX-211</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>690082-1</t>
+          <t>690064-3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ประชุม คุณท้าวเทียม</t>
+          <t>จีรวรรณ มณีโชติ</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>มีบุญ</t>
+          <t>ชาแนล</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3979,12 +4061,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3994,29 +4076,29 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DRX-151</t>
+          <t>DRX-212</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>690096-1</t>
+          <t>690064-4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>กฤตยา วิเชียรพาย</t>
+          <t>จีรวรรณ มณีโชติ</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ซาร่า</t>
+          <t>เนปจูน</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -4031,7 +4113,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4041,29 +4123,29 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DRX-161</t>
+          <t>DRX-214</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>690100-1</t>
+          <t>690064-6</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>พิสิทธิ์    สามกองงาม</t>
+          <t>จีรวรรณ มณีโชติ</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>กิมจิ</t>
+          <t>กาแฟ</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4073,12 +4155,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4088,29 +4170,29 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DRX-159</t>
+          <t>DRX-209</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>690100-2</t>
+          <t>690064-1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>พิสิทธิ์    สามกองงาม</t>
+          <t>จีรวรรณ มณีโชติ</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>โซจู</t>
+          <t>ลาคอส</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -4120,12 +4202,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4135,29 +4217,29 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DRX-163</t>
+          <t>DRX-213</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>690056-2</t>
+          <t>690064-5</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>อรธิมา เอกจีน</t>
+          <t>จีรวรรณ มณีโชติ</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>เฉาก๊วย</t>
+          <t>ปลาวาฬ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4172,7 +4254,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4182,29 +4264,29 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DRX-164</t>
+          <t>DRX-218</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>690056-3</t>
+          <t>690122-1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>อรธิมา เอกจีน</t>
+          <t>วิทวัส ศรีลำไย</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>พาดกลอน</t>
+          <t>โอริโอ้</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4214,12 +4296,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4229,44 +4311,44 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DRX-174</t>
+          <t>DRX-229</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>690056-4</t>
+          <t>690127-1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>อรธิมา เอกจีน</t>
+          <t>เจนจิรา</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>บี1</t>
+          <t>จัสติน</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
+          <t>เบญจมาศ</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ (DW)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4276,289 +4358,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-05-26 20:36:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>DRX-180</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>690042-2</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>วราฤทธิ์ บัวโต</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>ดั๊ก</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>drx</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>2026-05-26 20:36:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>DRX-172</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>690056-5</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>อรธิมา เอกจีน</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>บี2</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>drx</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>2026-05-26 20:36:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>DRX-191</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>690009-6</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>ธนาวดี เมธา</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>ปลาหมึก</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>drx</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>2026-05-26 20:36:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>DRX-210</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>690064-2</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>จีรวรรณ มณีโชติ</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>พลูโต</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>drx</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>2026-05-26 20:36:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>DRX-211</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>690064-3</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>จีรวรรณ มณีโชติ</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>ชาแนล</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>drx</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>2026-05-26 20:36:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>DRX-212</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>690064-4</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>จีรวรรณ มณีโชติ</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>เนปจูน</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>นารีรัตน์ ผลทิพย์</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>drx</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>2026-05-26 20:36:12</t>
+          <t>2026-05-27 20:15:06</t>
         </is>
       </c>
     </row>
@@ -4710,7 +4510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6749,7 +6549,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -6794,7 +6594,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -6839,7 +6639,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -6884,7 +6684,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -6929,7 +6729,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -7084,7 +6884,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -7129,7 +6929,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>NoLine</t>
+          <t>Expired</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -7758,6 +7558,331 @@
         </is>
       </c>
       <c r="P63" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>10037</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>690171-2</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>สุดารัตน์ โพธิ์ทอง</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ไดม่อน</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>นารีรัตน์ ผลทิพย์</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (3/3) + พิษสุนัขบ้า (2/2)) / ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>NoLine</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>10038</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>690171-1</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>สุดารัตน์ โพธิ์ทอง</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ดราก้อน (แพคเกจวัคซีน)</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>นารีรัตน์ ผลทิพย์</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ,หยอดยา/รับยา/ป้อนยา/ฉีดยาป้องกันปรสิตภายนอก / ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/3) +  พิษสุนัขบ้า (1/2))</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>NoLine</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>10039</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>690178-1</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ณิชจิรา เติมสินสวัสดิ์</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>มะยม (แพคเกจวัคซีน)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>นารีรัตน์ ผลทิพย์</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>ตรวจทั่วไป — ถ่ายพยาธิ / ฉีดวัคซีน — วัคซีนพิษสุนัขบ้า,วัคซีนไข้หัดและหวัดแมว (ไข้หัด (2/3) + พิษสุนัขบ้า (2/2))</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>NoLine</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>10040</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>690284-1</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>จันทนี เซี่ยงคิ้ว</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ชานม</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>สัตวแพทย์</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>ตรวจทั่วไป — ดูอาการ,รับยาต่อเนื่อง</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Ue95e6b9adfedfe87453d8d88c805be9a</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2026-05-27 18:00:03</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>10041</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>690136-1</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ลูกนัท</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>มีอาร์</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>สัตวแพทย์</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>ตรวจทั่วไป — ดูอาการ (+/- กระตุ้นวัคซีน รวม2/2 + RV2/2)</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>NoLine</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>10042</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>690298-1</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>กรรณิการ์ วุฒิกุล</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>มาตังค์</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>นารีรัตน์ ผลทิพย์</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>ตรวจทั่วไป — ดูอาการ (ตาบวม)</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>NoLine</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>drx</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>10043</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>690152-4</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ปวริศ มากสอน</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>บีน่า</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>นารีรัตน์ ผลทิพย์</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ตรวจทั่วไป — ดูอาการ (เท้าบวม)</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>NoLine</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
         <is>
           <t>drx</t>
         </is>
@@ -7785,7 +7910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12182,6 +12307,692 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:08</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>DRX_Sync</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>DRX:67</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:09</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>690001-1</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Ud4b955ac4ddd56e12f2ab3cbc77f790b</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:10</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>690001-1</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Ub52a3ad9704e3f5c3194c5cf96875084</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:11</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>690224-1</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>U319ce6867f8c2e421e72170330fca9ce</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:12</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>690287-2</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>U12d49c2dfd70e222ff4d4e5febe9a27a</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:13</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>690165-1</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>U767d6bba954a02bc3bd47fa2156cefb2</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:14</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>690284-1</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Ue95e6b9adfedfe87453d8d88c805be9a</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:15</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>690291-1</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>U85ffc0c0ed720e5aa118f80fe81e4f51</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:16</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>690131-2</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Ud3199338d71e5f310af197255682ff41</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:17</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>690157-1</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>U9d5f25862cbd9d2fe2c58bb5ba7c532f</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:18</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>690118-1</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Ub741455c24a2afcee792ea9d8af87077</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:18</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>690160-2</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>U4641000ef0dc24781745999e95de3998</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:19</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>690289-1</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>U7cc0f7ce8f6e545e67c7e77aa35db9ce</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:20</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>690299-3</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>U47aa79494e18e479471bae5f420f8caf</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:21</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>690084-2</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>U22ef391387145f0f1cfd0889a2e437f9</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:22</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>690189-1</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>U5d220d047421251dbe36331d61631e3a</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:23</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>690201-1</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>U835cf6a27aa276bd81a80630f363998b</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:05:25</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Queue_Build</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Queue+0</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:30:16</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>RegisterSibling</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>690299-1</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>U47aa79494e18e479471bae5f420f8caf</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>sibling HN → บราวนี่</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:30:25</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>DRX_Sync</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>DRX:67</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-05-27 13:00:02</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Queue_Build</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Queue+7</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-05-27 20:15:12</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>RegisterSibling</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>690084-3</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>U22ef391387145f0f1cfd0889a2e437f9</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>sibling HN → ชาไทย</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-05-27 20:15:22</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>DRX_Sync</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>DRX:61</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>